<commit_message>
fix: rename smu-kediri-sgi to sgi-kediri in masterlist and DB backup
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/CCTV_Master_List.xlsx
+++ b/CCTV_Master_List.xlsx
@@ -20,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -40,8 +40,20 @@
       <b val="1"/>
       <color rgb="00FFFFFF"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="11">
+  <fills count="12">
     <fill>
       <patternFill/>
     </fill>
@@ -93,6 +105,11 @@
         <fgColor rgb="00D9D9D9"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0037474F"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -120,7 +137,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -153,6 +170,24 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -519,7 +554,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P148"/>
+  <dimension ref="A1:P147"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -660,7 +695,7 @@
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>ame-krian</t>
+          <t>ame-gudang-krian</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
@@ -779,7 +814,7 @@
         </is>
       </c>
       <c r="P3" s="11" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
     </row>
     <row r="4">
@@ -1098,10 +1133,8 @@
           <t>unreachable</t>
         </is>
       </c>
-      <c r="P7" s="12" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="P7" s="12" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="8">
@@ -1180,10 +1213,8 @@
           <t>unreachable</t>
         </is>
       </c>
-      <c r="P8" s="12" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="P8" s="12" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="9">
@@ -1262,10 +1293,8 @@
           <t>unreachable</t>
         </is>
       </c>
-      <c r="P9" s="12" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="P9" s="12" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="10">
@@ -1344,10 +1373,8 @@
           <t>unreachable</t>
         </is>
       </c>
-      <c r="P10" s="12" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="P10" s="12" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="11">
@@ -1749,18 +1776,52 @@
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="H16" s="2" t="inlineStr"/>
-      <c r="I16" s="2" t="inlineStr"/>
-      <c r="J16" s="2" t="inlineStr"/>
-      <c r="K16" s="2" t="inlineStr"/>
-      <c r="L16" s="2" t="inlineStr"/>
-      <c r="M16" s="2" t="inlineStr"/>
-      <c r="N16" s="2" t="inlineStr"/>
-      <c r="O16" s="2" t="inlineStr"/>
-      <c r="P16" s="2" t="inlineStr"/>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>sgi-batulicin</t>
+        </is>
+      </c>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t>192.168.19.170</t>
+        </is>
+      </c>
+      <c r="J16" s="2" t="inlineStr">
+        <is>
+          <t>80</t>
+        </is>
+      </c>
+      <c r="K16" s="2" t="inlineStr">
+        <is>
+          <t>554</t>
+        </is>
+      </c>
+      <c r="L16" s="2" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+      <c r="M16" s="2" t="inlineStr">
+        <is>
+          <t>123456</t>
+        </is>
+      </c>
+      <c r="N16" s="2" t="inlineStr">
+        <is>
+          <t>acti_snvr</t>
+        </is>
+      </c>
+      <c r="O16" s="2" t="inlineStr">
+        <is>
+          <t>synced</t>
+        </is>
+      </c>
+      <c r="P16" s="2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -1884,10 +1945,8 @@
           <t>unreachable</t>
         </is>
       </c>
-      <c r="P18" s="12" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="P18" s="12" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="19">
@@ -2551,7 +2610,7 @@
         </is>
       </c>
       <c r="P28" s="11" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="29">
@@ -2769,7 +2828,7 @@
         </is>
       </c>
       <c r="P32" s="11" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="33">
@@ -3055,7 +3114,7 @@
         </is>
       </c>
       <c r="P36" s="11" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="37">
@@ -3260,10 +3319,8 @@
           <t>unreachable</t>
         </is>
       </c>
-      <c r="P39" s="12" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="P39" s="12" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="40">
@@ -3434,10 +3491,8 @@
           <t>unreachable</t>
         </is>
       </c>
-      <c r="P42" s="12" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="P42" s="12" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="43">
@@ -3826,10 +3881,8 @@
           <t>unreachable</t>
         </is>
       </c>
-      <c r="P49" s="12" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="P49" s="12" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="50">
@@ -3865,18 +3918,52 @@
       </c>
       <c r="G50" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="H50" s="2" t="inlineStr"/>
-      <c r="I50" s="2" t="inlineStr"/>
-      <c r="J50" s="2" t="inlineStr"/>
-      <c r="K50" s="2" t="inlineStr"/>
-      <c r="L50" s="2" t="inlineStr"/>
-      <c r="M50" s="2" t="inlineStr"/>
-      <c r="N50" s="2" t="inlineStr"/>
-      <c r="O50" s="2" t="inlineStr"/>
-      <c r="P50" s="2" t="inlineStr"/>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="H50" s="2" t="inlineStr">
+        <is>
+          <t>sgi-sampit</t>
+        </is>
+      </c>
+      <c r="I50" s="2" t="inlineStr">
+        <is>
+          <t>10.70.130.200</t>
+        </is>
+      </c>
+      <c r="J50" s="2" t="inlineStr">
+        <is>
+          <t>80</t>
+        </is>
+      </c>
+      <c r="K50" s="2" t="inlineStr">
+        <is>
+          <t>554</t>
+        </is>
+      </c>
+      <c r="L50" s="2" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+      <c r="M50" s="2" t="inlineStr">
+        <is>
+          <t>1234qwer</t>
+        </is>
+      </c>
+      <c r="N50" s="2" t="inlineStr">
+        <is>
+          <t>hikvision</t>
+        </is>
+      </c>
+      <c r="O50" s="2" t="inlineStr">
+        <is>
+          <t>synced</t>
+        </is>
+      </c>
+      <c r="P50" s="2" t="n">
+        <v>12</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -4046,10 +4133,8 @@
           <t>unreachable</t>
         </is>
       </c>
-      <c r="P53" s="12" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="P53" s="12" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="54">
@@ -4187,7 +4272,7 @@
       </c>
       <c r="I56" s="3" t="inlineStr">
         <is>
-          <t>192.168.18.200</t>
+          <t>192.168.18.170</t>
         </is>
       </c>
       <c r="J56" s="3" t="inlineStr">
@@ -4212,18 +4297,16 @@
       </c>
       <c r="N56" s="3" t="inlineStr">
         <is>
-          <t>hikvision</t>
+          <t>acti_snvr</t>
         </is>
       </c>
       <c r="O56" s="12" t="inlineStr">
         <is>
-          <t>unreachable</t>
-        </is>
-      </c>
-      <c r="P56" s="12" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+          <t>synced</t>
+        </is>
+      </c>
+      <c r="P56" s="12" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="57">
@@ -4302,10 +4385,8 @@
           <t>unreachable</t>
         </is>
       </c>
-      <c r="P57" s="12" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="P57" s="12" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="58">
@@ -4636,10 +4717,8 @@
           <t>auth_error</t>
         </is>
       </c>
-      <c r="P62" s="13" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="P62" s="13" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="63">
@@ -5017,7 +5096,7 @@
         </is>
       </c>
       <c r="P68" s="11" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="69">
@@ -5096,10 +5175,8 @@
           <t>failed</t>
         </is>
       </c>
-      <c r="P69" s="13" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="P69" s="13" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="70">
@@ -5140,7 +5217,7 @@
       </c>
       <c r="H70" s="2" t="inlineStr">
         <is>
-          <t>sig-cikande</t>
+          <t>sgi-cikande</t>
         </is>
       </c>
       <c r="I70" s="2" t="inlineStr">
@@ -5215,18 +5292,52 @@
       </c>
       <c r="G71" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="H71" s="2" t="inlineStr"/>
-      <c r="I71" s="2" t="inlineStr"/>
-      <c r="J71" s="2" t="inlineStr"/>
-      <c r="K71" s="2" t="inlineStr"/>
-      <c r="L71" s="2" t="inlineStr"/>
-      <c r="M71" s="2" t="inlineStr"/>
-      <c r="N71" s="2" t="inlineStr"/>
-      <c r="O71" s="2" t="inlineStr"/>
-      <c r="P71" s="2" t="inlineStr"/>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="H71" s="2" t="inlineStr">
+        <is>
+          <t>sig-cikarang-cbc</t>
+        </is>
+      </c>
+      <c r="I71" s="2" t="inlineStr">
+        <is>
+          <t>192.168.67.200</t>
+        </is>
+      </c>
+      <c r="J71" s="2" t="inlineStr">
+        <is>
+          <t>80</t>
+        </is>
+      </c>
+      <c r="K71" s="2" t="inlineStr">
+        <is>
+          <t>554</t>
+        </is>
+      </c>
+      <c r="L71" s="2" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+      <c r="M71" s="2" t="inlineStr">
+        <is>
+          <t>P4SSW0RD</t>
+        </is>
+      </c>
+      <c r="N71" s="2" t="inlineStr">
+        <is>
+          <t>hilook</t>
+        </is>
+      </c>
+      <c r="O71" s="2" t="inlineStr">
+        <is>
+          <t>unreachable</t>
+        </is>
+      </c>
+      <c r="P71" s="2" t="n">
+        <v>14</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -5266,7 +5377,7 @@
       </c>
       <c r="H72" s="2" t="inlineStr">
         <is>
-          <t>sig-cilamaya</t>
+          <t>smt-cilamaya</t>
         </is>
       </c>
       <c r="I72" s="2" t="inlineStr">
@@ -5678,7 +5789,7 @@
       </c>
       <c r="H78" s="2" t="inlineStr">
         <is>
-          <t>sig-lampung-tengah</t>
+          <t>sig-lampung-3</t>
         </is>
       </c>
       <c r="I78" s="2" t="inlineStr">
@@ -5922,10 +6033,8 @@
           <t>unreachable</t>
         </is>
       </c>
-      <c r="P81" s="12" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="P81" s="12" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="82">
@@ -6176,10 +6285,8 @@
           <t>unreachable</t>
         </is>
       </c>
-      <c r="P85" s="12" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="P85" s="12" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="86">
@@ -6258,10 +6365,8 @@
           <t>unreachable</t>
         </is>
       </c>
-      <c r="P86" s="12" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="P86" s="12" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="87">
@@ -8184,10 +8289,8 @@
           <t>unreachable</t>
         </is>
       </c>
-      <c r="P123" s="12" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="P123" s="12" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="124">
@@ -8361,7 +8464,7 @@
         </is>
       </c>
       <c r="P126" s="11" t="n">
-        <v>0</v>
+        <v>23</v>
       </c>
     </row>
     <row r="127">
@@ -8424,10 +8527,8 @@
           <t>unreachable</t>
         </is>
       </c>
-      <c r="P127" s="12" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="P127" s="12" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="128">
@@ -8910,10 +9011,8 @@
           <t>unreachable</t>
         </is>
       </c>
-      <c r="P136" s="12" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="P136" s="12" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="137">
@@ -9232,10 +9331,8 @@
           <t>auth_error</t>
         </is>
       </c>
-      <c r="P141" s="13" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="P141" s="13" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="142">
@@ -9370,7 +9467,7 @@
       <c r="A144" s="5" t="inlineStr"/>
       <c r="B144" s="5" t="inlineStr">
         <is>
-          <t>Sig Cikarang Cbc</t>
+          <t>Sig Kendal 1</t>
         </is>
       </c>
       <c r="C144" s="5" t="inlineStr"/>
@@ -9388,12 +9485,12 @@
       </c>
       <c r="H144" s="5" t="inlineStr">
         <is>
-          <t>sig-cikarang-cbc</t>
+          <t>sig-kendal-1</t>
         </is>
       </c>
       <c r="I144" s="5" t="inlineStr">
         <is>
-          <t>192.168.67.200</t>
+          <t>192.168.2.100</t>
         </is>
       </c>
       <c r="J144" s="5" t="inlineStr">
@@ -9413,30 +9510,28 @@
       </c>
       <c r="M144" s="5" t="inlineStr">
         <is>
-          <t>P4SSW0RD</t>
+          <t>Indogas*19#</t>
         </is>
       </c>
       <c r="N144" s="5" t="inlineStr">
         <is>
-          <t>hilook</t>
-        </is>
-      </c>
-      <c r="O144" s="12" t="inlineStr">
-        <is>
-          <t>unreachable</t>
-        </is>
-      </c>
-      <c r="P144" s="12" t="inlineStr">
-        <is>
-          <t>14</t>
-        </is>
+          <t>hikvision</t>
+        </is>
+      </c>
+      <c r="O144" s="11" t="inlineStr">
+        <is>
+          <t>synced</t>
+        </is>
+      </c>
+      <c r="P144" s="11" t="n">
+        <v>26</v>
       </c>
     </row>
     <row r="145">
       <c r="A145" s="5" t="inlineStr"/>
       <c r="B145" s="5" t="inlineStr">
         <is>
-          <t>Sig Kendal 1</t>
+          <t>Sig Rungkut Sier</t>
         </is>
       </c>
       <c r="C145" s="5" t="inlineStr"/>
@@ -9454,12 +9549,12 @@
       </c>
       <c r="H145" s="5" t="inlineStr">
         <is>
-          <t>sig-kendal-1</t>
+          <t>sig-rungkut-sier</t>
         </is>
       </c>
       <c r="I145" s="5" t="inlineStr">
         <is>
-          <t>192.168.2.100</t>
+          <t>10.70.90.200</t>
         </is>
       </c>
       <c r="J145" s="5" t="inlineStr">
@@ -9479,12 +9574,12 @@
       </c>
       <c r="M145" s="5" t="inlineStr">
         <is>
-          <t>Indogas*19#</t>
+          <t>123456</t>
         </is>
       </c>
       <c r="N145" s="5" t="inlineStr">
         <is>
-          <t>hikvision</t>
+          <t>acti_snvr</t>
         </is>
       </c>
       <c r="O145" s="11" t="inlineStr">
@@ -9493,14 +9588,14 @@
         </is>
       </c>
       <c r="P145" s="11" t="n">
-        <v>26</v>
+        <v>0</v>
       </c>
     </row>
     <row r="146">
       <c r="A146" s="5" t="inlineStr"/>
       <c r="B146" s="5" t="inlineStr">
         <is>
-          <t>Sig Rungkut Sier</t>
+          <t>SGI Kediri</t>
         </is>
       </c>
       <c r="C146" s="5" t="inlineStr"/>
@@ -9518,12 +9613,12 @@
       </c>
       <c r="H146" s="5" t="inlineStr">
         <is>
-          <t>sig-rungkut-sier</t>
+          <t>sgi-kediri</t>
         </is>
       </c>
       <c r="I146" s="5" t="inlineStr">
         <is>
-          <t>10.70.90.200</t>
+          <t>10.70.137.201</t>
         </is>
       </c>
       <c r="J146" s="5" t="inlineStr">
@@ -9543,20 +9638,20 @@
       </c>
       <c r="M146" s="5" t="inlineStr">
         <is>
-          <t>123456</t>
+          <t>Aremania87</t>
         </is>
       </c>
       <c r="N146" s="5" t="inlineStr">
         <is>
-          <t>acti_snvr</t>
-        </is>
-      </c>
-      <c r="O146" s="11" t="inlineStr">
-        <is>
-          <t>synced</t>
-        </is>
-      </c>
-      <c r="P146" s="11" t="n">
+          <t>hikvision</t>
+        </is>
+      </c>
+      <c r="O146" s="12" t="inlineStr">
+        <is>
+          <t>unreachable</t>
+        </is>
+      </c>
+      <c r="P146" s="12" t="n">
         <v>0</v>
       </c>
     </row>
@@ -9564,7 +9659,7 @@
       <c r="A147" s="5" t="inlineStr"/>
       <c r="B147" s="5" t="inlineStr">
         <is>
-          <t>Smu Kediri Sgi</t>
+          <t>Smu Sidoarjo Sgi</t>
         </is>
       </c>
       <c r="C147" s="5" t="inlineStr"/>
@@ -9582,12 +9677,12 @@
       </c>
       <c r="H147" s="5" t="inlineStr">
         <is>
-          <t>smu-kediri-sgi</t>
+          <t>smu-sidoarjo-sgi</t>
         </is>
       </c>
       <c r="I147" s="5" t="inlineStr">
         <is>
-          <t>10.70.137.201</t>
+          <t>10.70.140.200</t>
         </is>
       </c>
       <c r="J147" s="5" t="inlineStr">
@@ -9607,12 +9702,12 @@
       </c>
       <c r="M147" s="5" t="inlineStr">
         <is>
-          <t>Aremania87</t>
+          <t>123456</t>
         </is>
       </c>
       <c r="N147" s="5" t="inlineStr">
         <is>
-          <t>hikvision</t>
+          <t>acti_snvr</t>
         </is>
       </c>
       <c r="O147" s="12" t="inlineStr">
@@ -9620,76 +9715,8 @@
           <t>unreachable</t>
         </is>
       </c>
-      <c r="P147" s="12" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-    </row>
-    <row r="148">
-      <c r="A148" s="5" t="inlineStr"/>
-      <c r="B148" s="5" t="inlineStr">
-        <is>
-          <t>Smu Sidoarjo Sgi</t>
-        </is>
-      </c>
-      <c r="C148" s="5" t="inlineStr"/>
-      <c r="D148" s="5" t="inlineStr"/>
-      <c r="E148" s="5" t="inlineStr"/>
-      <c r="F148" s="5" t="inlineStr">
-        <is>
-          <t>Not in SHE Request</t>
-        </is>
-      </c>
-      <c r="G148" s="5" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="H148" s="5" t="inlineStr">
-        <is>
-          <t>smu-sidoarjo-sgi</t>
-        </is>
-      </c>
-      <c r="I148" s="5" t="inlineStr">
-        <is>
-          <t>10.70.140.200</t>
-        </is>
-      </c>
-      <c r="J148" s="5" t="inlineStr">
-        <is>
-          <t>80</t>
-        </is>
-      </c>
-      <c r="K148" s="5" t="inlineStr">
-        <is>
-          <t>554</t>
-        </is>
-      </c>
-      <c r="L148" s="5" t="inlineStr">
-        <is>
-          <t>admin</t>
-        </is>
-      </c>
-      <c r="M148" s="5" t="inlineStr">
-        <is>
-          <t>123456</t>
-        </is>
-      </c>
-      <c r="N148" s="5" t="inlineStr">
-        <is>
-          <t>acti_snvr</t>
-        </is>
-      </c>
-      <c r="O148" s="12" t="inlineStr">
-        <is>
-          <t>unreachable</t>
-        </is>
-      </c>
-      <c r="P148" s="12" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="P147" s="12" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -9704,70 +9731,262 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B5"/>
+  <dimension ref="A1:B23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="55" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="72" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="6" t="inlineStr">
-        <is>
-          <t>Color</t>
-        </is>
-      </c>
-      <c r="B1" s="6" t="inlineStr">
-        <is>
-          <t>Meaning</t>
+      <c r="A1" s="15" t="inlineStr">
+        <is>
+          <t>ROW COLOR</t>
+        </is>
+      </c>
+      <c r="B1" s="15" t="inlineStr">
+        <is>
+          <t>MEANING</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="7" t="inlineStr">
+      <c r="A2" s="16" t="inlineStr">
+        <is>
+          <t>Pink / Light Red</t>
+        </is>
+      </c>
+      <c r="B2" s="17" t="inlineStr">
+        <is>
+          <t>Requested by SHE — site is in the SHE access request list</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="18" t="inlineStr">
         <is>
           <t>Green</t>
         </is>
       </c>
-      <c r="B2" s="7" t="inlineStr">
-        <is>
-          <t>In SHE request list AND in DB (configured)</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="8" t="inlineStr">
-        <is>
-          <t>Red</t>
-        </is>
-      </c>
-      <c r="B3" s="8" t="inlineStr">
-        <is>
-          <t>In SHE request list but NOT in DB (needs to be added)</t>
+      <c r="B3" s="17" t="inlineStr">
+        <is>
+          <t>Active &amp; synced — NVR is reachable and confirmed in DB</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="9" t="inlineStr">
-        <is>
-          <t>Yellow</t>
-        </is>
-      </c>
-      <c r="B4" s="9" t="inlineStr">
-        <is>
-          <t>In DB but NOT in SHE request list (extra sites)</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="10" t="inlineStr">
-        <is>
-          <t>Pink</t>
-        </is>
-      </c>
-      <c r="B5" s="10" t="inlineStr">
-        <is>
-          <t>NVR is unreachable</t>
+      <c r="A4" s="19" t="inlineStr">
+        <is>
+          <t>Yellow / Amber</t>
+        </is>
+      </c>
+      <c r="B4" s="17" t="inlineStr">
+        <is>
+          <t>Not in SHE request — site is in DB but was not requested by SHE</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="15" t="inlineStr">
+        <is>
+          <t>SYNC STATUS</t>
+        </is>
+      </c>
+      <c r="B6" s="15" t="inlineStr">
+        <is>
+          <t>MEANING</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="20" t="inlineStr">
+        <is>
+          <t>synced</t>
+        </is>
+      </c>
+      <c r="B7" s="17" t="inlineStr">
+        <is>
+          <t>NVR is reachable and device info has been retrieved successfully</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="20" t="inlineStr">
+        <is>
+          <t>unreachable</t>
+        </is>
+      </c>
+      <c r="B8" s="17" t="inlineStr">
+        <is>
+          <t>NVR did not respond within timeout — network/VPN issue or device offline</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="20" t="inlineStr">
+        <is>
+          <t>auth_error</t>
+        </is>
+      </c>
+      <c r="B9" s="17" t="inlineStr">
+        <is>
+          <t>NVR responded but login failed — credentials need to be updated</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="20" t="inlineStr">
+        <is>
+          <t>failed</t>
+        </is>
+      </c>
+      <c r="B10" s="17" t="inlineStr">
+        <is>
+          <t>NVR responded but ISAPI returned an error — possibly wrong vendor type</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="20" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="B11" s="17" t="inlineStr">
+        <is>
+          <t>Not yet probed since last import</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="15" t="inlineStr">
+        <is>
+          <t>COLUMN</t>
+        </is>
+      </c>
+      <c r="B13" s="15" t="inlineStr">
+        <is>
+          <t>MEANING</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="20" t="inlineStr">
+        <is>
+          <t>Plant Code</t>
+        </is>
+      </c>
+      <c r="B14" s="17" t="inlineStr">
+        <is>
+          <t>Epicor plant code (e.g. SGI046)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="20" t="inlineStr">
+        <is>
+          <t>Site Name</t>
+        </is>
+      </c>
+      <c r="B15" s="17" t="inlineStr">
+        <is>
+          <t>Official site name used in SHE/Epicor</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="20" t="inlineStr">
+        <is>
+          <t>Company</t>
+        </is>
+      </c>
+      <c r="B16" s="17" t="inlineStr">
+        <is>
+          <t>Legal entity (SGI, SIG, AME, SMT, etc.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="20" t="inlineStr">
+        <is>
+          <t>SHE Status</t>
+        </is>
+      </c>
+      <c r="B17" s="17" t="inlineStr">
+        <is>
+          <t>Whether SHE has requested CCTV access for this site</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="20" t="inlineStr">
+        <is>
+          <t>In DB</t>
+        </is>
+      </c>
+      <c r="B18" s="17" t="inlineStr">
+        <is>
+          <t>YES = NVR is registered in the CCTV system database</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="20" t="inlineStr">
+        <is>
+          <t>DB Code</t>
+        </is>
+      </c>
+      <c r="B19" s="17" t="inlineStr">
+        <is>
+          <t>Unique identifier used in the CCTV system (slug format)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="20" t="inlineStr">
+        <is>
+          <t>NVR IP</t>
+        </is>
+      </c>
+      <c r="B20" s="17" t="inlineStr">
+        <is>
+          <t>IP address of the NVR on the internal network</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="20" t="inlineStr">
+        <is>
+          <t>Vendor</t>
+        </is>
+      </c>
+      <c r="B21" s="17" t="inlineStr">
+        <is>
+          <t>NVR brand/protocol: hikvision | acti_snvr | uniview | hilook</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="20" t="inlineStr">
+        <is>
+          <t>Sync Status</t>
+        </is>
+      </c>
+      <c r="B22" s="17" t="inlineStr">
+        <is>
+          <t>Result of last probe (see Sync Status table above)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="20" t="inlineStr">
+        <is>
+          <t>Channels</t>
+        </is>
+      </c>
+      <c r="B23" s="17" t="inlineStr">
+        <is>
+          <t>Number of camera channels discovered on this NVR</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: add Playback Test sheet to master list
Results for 52 NVRs tested 2026-06-23 ch1 10:00-10:01 WIB:
24 works (Hikvision/Hilook), 26 no recording, 2 Uniview unsupported

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/CCTV_Master_List.xlsx
+++ b/CCTV_Master_List.xlsx
@@ -9,6 +9,7 @@
   <sheets>
     <sheet name="CCTV Master List" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Legend" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Playback Test" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'CCTV Master List'!$A$1:$P$1</definedName>
@@ -20,7 +21,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="7">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -52,8 +53,17 @@
     <font>
       <sz val="10"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="13"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="12">
+  <fills count="17">
     <fill>
       <patternFill/>
     </fill>
@@ -110,8 +120,33 @@
         <fgColor rgb="0037474F"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="002E4057"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="004472C4"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9F0D9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF5CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFD9D9"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -133,11 +168,17 @@
         <color rgb="00CCCCCC"/>
       </bottom>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -187,6 +228,69 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="12" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="13" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="16" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="16" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="16" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -9993,4 +10097,1370 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E55"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="48" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="21" t="inlineStr">
+        <is>
+          <t>Playback Test Results — 2026-06-23, Channel 1, 10:00–10:01 WIB</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="18" customHeight="1">
+      <c r="A2" s="22" t="inlineStr">
+        <is>
+          <t>52 NVRs tested  |  24 Works  |  26 No Recording  |  2 API Not Supported</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="20" customHeight="1">
+      <c r="A3" s="23" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B3" s="23" t="inlineStr">
+        <is>
+          <t>Site Code</t>
+        </is>
+      </c>
+      <c r="C3" s="23" t="inlineStr">
+        <is>
+          <t>Vendor</t>
+        </is>
+      </c>
+      <c r="D3" s="23" t="inlineStr">
+        <is>
+          <t>Playback Status</t>
+        </is>
+      </c>
+      <c r="E3" s="23" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="B4" s="25" t="inlineStr">
+        <is>
+          <t>arohera-lt3</t>
+        </is>
+      </c>
+      <c r="C4" s="25" t="inlineStr">
+        <is>
+          <t>Hikvision</t>
+        </is>
+      </c>
+      <c r="D4" s="25" t="inlineStr">
+        <is>
+          <t>✅ Works</t>
+        </is>
+      </c>
+      <c r="E4" s="26" t="inlineStr">
+        <is>
+          <t>1 segment found</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="27" t="n">
+        <v>2</v>
+      </c>
+      <c r="B5" s="28" t="inlineStr">
+        <is>
+          <t>depo-pangkalan-bun</t>
+        </is>
+      </c>
+      <c r="C5" s="28" t="inlineStr">
+        <is>
+          <t>Hikvision</t>
+        </is>
+      </c>
+      <c r="D5" s="28" t="inlineStr">
+        <is>
+          <t>✅ Works</t>
+        </is>
+      </c>
+      <c r="E5" s="29" t="inlineStr">
+        <is>
+          <t>1 segment found</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="24" t="n">
+        <v>3</v>
+      </c>
+      <c r="B6" s="25" t="inlineStr">
+        <is>
+          <t>depo-purwodadi</t>
+        </is>
+      </c>
+      <c r="C6" s="25" t="inlineStr">
+        <is>
+          <t>Hikvision</t>
+        </is>
+      </c>
+      <c r="D6" s="25" t="inlineStr">
+        <is>
+          <t>✅ Works</t>
+        </is>
+      </c>
+      <c r="E6" s="26" t="inlineStr">
+        <is>
+          <t>1 segment found</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="27" t="n">
+        <v>4</v>
+      </c>
+      <c r="B7" s="28" t="inlineStr">
+        <is>
+          <t>depo-rembang</t>
+        </is>
+      </c>
+      <c r="C7" s="28" t="inlineStr">
+        <is>
+          <t>Hikvision</t>
+        </is>
+      </c>
+      <c r="D7" s="28" t="inlineStr">
+        <is>
+          <t>✅ Works</t>
+        </is>
+      </c>
+      <c r="E7" s="29" t="inlineStr">
+        <is>
+          <t>1 segment found</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="24" t="n">
+        <v>5</v>
+      </c>
+      <c r="B8" s="25" t="inlineStr">
+        <is>
+          <t>ho-sby-lantai-15</t>
+        </is>
+      </c>
+      <c r="C8" s="25" t="inlineStr">
+        <is>
+          <t>Hikvision</t>
+        </is>
+      </c>
+      <c r="D8" s="25" t="inlineStr">
+        <is>
+          <t>✅ Works</t>
+        </is>
+      </c>
+      <c r="E8" s="26" t="inlineStr">
+        <is>
+          <t>1 segment found</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="27" t="n">
+        <v>6</v>
+      </c>
+      <c r="B9" s="28" t="inlineStr">
+        <is>
+          <t>satoe</t>
+        </is>
+      </c>
+      <c r="C9" s="28" t="inlineStr">
+        <is>
+          <t>Hikvision</t>
+        </is>
+      </c>
+      <c r="D9" s="28" t="inlineStr">
+        <is>
+          <t>✅ Works</t>
+        </is>
+      </c>
+      <c r="E9" s="29" t="inlineStr">
+        <is>
+          <t>1 segment found</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="24" t="n">
+        <v>7</v>
+      </c>
+      <c r="B10" s="25" t="inlineStr">
+        <is>
+          <t>sgi-bandung</t>
+        </is>
+      </c>
+      <c r="C10" s="25" t="inlineStr">
+        <is>
+          <t>Hikvision</t>
+        </is>
+      </c>
+      <c r="D10" s="25" t="inlineStr">
+        <is>
+          <t>✅ Works</t>
+        </is>
+      </c>
+      <c r="E10" s="26" t="inlineStr">
+        <is>
+          <t>1 segment found</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="27" t="n">
+        <v>8</v>
+      </c>
+      <c r="B11" s="28" t="inlineStr">
+        <is>
+          <t>sgi-batam</t>
+        </is>
+      </c>
+      <c r="C11" s="28" t="inlineStr">
+        <is>
+          <t>Hikvision</t>
+        </is>
+      </c>
+      <c r="D11" s="28" t="inlineStr">
+        <is>
+          <t>✅ Works</t>
+        </is>
+      </c>
+      <c r="E11" s="29" t="inlineStr">
+        <is>
+          <t>1 segment found</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="24" t="n">
+        <v>9</v>
+      </c>
+      <c r="B12" s="25" t="inlineStr">
+        <is>
+          <t>sgi-batam-2</t>
+        </is>
+      </c>
+      <c r="C12" s="25" t="inlineStr">
+        <is>
+          <t>Hikvision</t>
+        </is>
+      </c>
+      <c r="D12" s="25" t="inlineStr">
+        <is>
+          <t>✅ Works</t>
+        </is>
+      </c>
+      <c r="E12" s="26" t="inlineStr">
+        <is>
+          <t>1 segment found</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="27" t="n">
+        <v>10</v>
+      </c>
+      <c r="B13" s="28" t="inlineStr">
+        <is>
+          <t>sgi-cikande</t>
+        </is>
+      </c>
+      <c r="C13" s="28" t="inlineStr">
+        <is>
+          <t>Hikvision</t>
+        </is>
+      </c>
+      <c r="D13" s="28" t="inlineStr">
+        <is>
+          <t>✅ Works</t>
+        </is>
+      </c>
+      <c r="E13" s="29" t="inlineStr">
+        <is>
+          <t>1 segment found</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="24" t="n">
+        <v>11</v>
+      </c>
+      <c r="B14" s="25" t="inlineStr">
+        <is>
+          <t>sgi-cikupa</t>
+        </is>
+      </c>
+      <c r="C14" s="25" t="inlineStr">
+        <is>
+          <t>Hikvision</t>
+        </is>
+      </c>
+      <c r="D14" s="25" t="inlineStr">
+        <is>
+          <t>✅ Works</t>
+        </is>
+      </c>
+      <c r="E14" s="26" t="inlineStr">
+        <is>
+          <t>1 segment found</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="27" t="n">
+        <v>12</v>
+      </c>
+      <c r="B15" s="28" t="inlineStr">
+        <is>
+          <t>sgi-lubuk-gaung-dumai</t>
+        </is>
+      </c>
+      <c r="C15" s="28" t="inlineStr">
+        <is>
+          <t>Hikvision</t>
+        </is>
+      </c>
+      <c r="D15" s="28" t="inlineStr">
+        <is>
+          <t>✅ Works</t>
+        </is>
+      </c>
+      <c r="E15" s="29" t="inlineStr">
+        <is>
+          <t>1 segment found</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="24" t="n">
+        <v>13</v>
+      </c>
+      <c r="B16" s="25" t="inlineStr">
+        <is>
+          <t>sgi-rantau-prapat</t>
+        </is>
+      </c>
+      <c r="C16" s="25" t="inlineStr">
+        <is>
+          <t>Hikvision</t>
+        </is>
+      </c>
+      <c r="D16" s="25" t="inlineStr">
+        <is>
+          <t>✅ Works</t>
+        </is>
+      </c>
+      <c r="E16" s="26" t="inlineStr">
+        <is>
+          <t>1 segment found</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="27" t="n">
+        <v>14</v>
+      </c>
+      <c r="B17" s="28" t="inlineStr">
+        <is>
+          <t>sgi-tebing-tinggi</t>
+        </is>
+      </c>
+      <c r="C17" s="28" t="inlineStr">
+        <is>
+          <t>Hikvision</t>
+        </is>
+      </c>
+      <c r="D17" s="28" t="inlineStr">
+        <is>
+          <t>✅ Works</t>
+        </is>
+      </c>
+      <c r="E17" s="29" t="inlineStr">
+        <is>
+          <t>1 segment found</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="24" t="n">
+        <v>15</v>
+      </c>
+      <c r="B18" s="25" t="inlineStr">
+        <is>
+          <t>sig-baturaja</t>
+        </is>
+      </c>
+      <c r="C18" s="25" t="inlineStr">
+        <is>
+          <t>Hikvision</t>
+        </is>
+      </c>
+      <c r="D18" s="25" t="inlineStr">
+        <is>
+          <t>✅ Works</t>
+        </is>
+      </c>
+      <c r="E18" s="26" t="inlineStr">
+        <is>
+          <t>1 segment found</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="27" t="n">
+        <v>16</v>
+      </c>
+      <c r="B19" s="28" t="inlineStr">
+        <is>
+          <t>sig-kendal</t>
+        </is>
+      </c>
+      <c r="C19" s="28" t="inlineStr">
+        <is>
+          <t>Hikvision</t>
+        </is>
+      </c>
+      <c r="D19" s="28" t="inlineStr">
+        <is>
+          <t>✅ Works</t>
+        </is>
+      </c>
+      <c r="E19" s="29" t="inlineStr">
+        <is>
+          <t>1 segment found</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="24" t="n">
+        <v>17</v>
+      </c>
+      <c r="B20" s="25" t="inlineStr">
+        <is>
+          <t>sig-kendal-1</t>
+        </is>
+      </c>
+      <c r="C20" s="25" t="inlineStr">
+        <is>
+          <t>Hikvision</t>
+        </is>
+      </c>
+      <c r="D20" s="25" t="inlineStr">
+        <is>
+          <t>✅ Works</t>
+        </is>
+      </c>
+      <c r="E20" s="26" t="inlineStr">
+        <is>
+          <t>1 segment found</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="27" t="n">
+        <v>18</v>
+      </c>
+      <c r="B21" s="28" t="inlineStr">
+        <is>
+          <t>sig-lampung-3</t>
+        </is>
+      </c>
+      <c r="C21" s="28" t="inlineStr">
+        <is>
+          <t>Hikvision</t>
+        </is>
+      </c>
+      <c r="D21" s="28" t="inlineStr">
+        <is>
+          <t>✅ Works</t>
+        </is>
+      </c>
+      <c r="E21" s="29" t="inlineStr">
+        <is>
+          <t>1 segment found</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="24" t="n">
+        <v>19</v>
+      </c>
+      <c r="B22" s="25" t="inlineStr">
+        <is>
+          <t>sig-lampung-ultimate</t>
+        </is>
+      </c>
+      <c r="C22" s="25" t="inlineStr">
+        <is>
+          <t>Hikvision</t>
+        </is>
+      </c>
+      <c r="D22" s="25" t="inlineStr">
+        <is>
+          <t>✅ Works</t>
+        </is>
+      </c>
+      <c r="E22" s="26" t="inlineStr">
+        <is>
+          <t>1 segment found</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="27" t="n">
+        <v>20</v>
+      </c>
+      <c r="B23" s="28" t="inlineStr">
+        <is>
+          <t>sig-medan</t>
+        </is>
+      </c>
+      <c r="C23" s="28" t="inlineStr">
+        <is>
+          <t>Hikvision</t>
+        </is>
+      </c>
+      <c r="D23" s="28" t="inlineStr">
+        <is>
+          <t>✅ Works</t>
+        </is>
+      </c>
+      <c r="E23" s="29" t="inlineStr">
+        <is>
+          <t>1 segment found</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="24" t="n">
+        <v>21</v>
+      </c>
+      <c r="B24" s="25" t="inlineStr">
+        <is>
+          <t>sig-medan-plant</t>
+        </is>
+      </c>
+      <c r="C24" s="25" t="inlineStr">
+        <is>
+          <t>Hikvision</t>
+        </is>
+      </c>
+      <c r="D24" s="25" t="inlineStr">
+        <is>
+          <t>✅ Works</t>
+        </is>
+      </c>
+      <c r="E24" s="26" t="inlineStr">
+        <is>
+          <t>1 segment found</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="27" t="n">
+        <v>22</v>
+      </c>
+      <c r="B25" s="28" t="inlineStr">
+        <is>
+          <t>sig-pulogadung</t>
+        </is>
+      </c>
+      <c r="C25" s="28" t="inlineStr">
+        <is>
+          <t>Hilook</t>
+        </is>
+      </c>
+      <c r="D25" s="28" t="inlineStr">
+        <is>
+          <t>✅ Works</t>
+        </is>
+      </c>
+      <c r="E25" s="29" t="inlineStr">
+        <is>
+          <t>1 segment found</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="24" t="n">
+        <v>23</v>
+      </c>
+      <c r="B26" s="25" t="inlineStr">
+        <is>
+          <t>sig-subang-pabrikan-pos</t>
+        </is>
+      </c>
+      <c r="C26" s="25" t="inlineStr">
+        <is>
+          <t>Hikvision</t>
+        </is>
+      </c>
+      <c r="D26" s="25" t="inlineStr">
+        <is>
+          <t>✅ Works</t>
+        </is>
+      </c>
+      <c r="E26" s="26" t="inlineStr">
+        <is>
+          <t>1 segment found</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="27" t="n">
+        <v>24</v>
+      </c>
+      <c r="B27" s="28" t="inlineStr">
+        <is>
+          <t>smt-cilamaya</t>
+        </is>
+      </c>
+      <c r="C27" s="28" t="inlineStr">
+        <is>
+          <t>Hikvision</t>
+        </is>
+      </c>
+      <c r="D27" s="28" t="inlineStr">
+        <is>
+          <t>✅ Works</t>
+        </is>
+      </c>
+      <c r="E27" s="29" t="inlineStr">
+        <is>
+          <t>1 segment found</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="30" t="n">
+        <v>25</v>
+      </c>
+      <c r="B28" s="31" t="inlineStr">
+        <is>
+          <t>sgi-cilegon</t>
+        </is>
+      </c>
+      <c r="C28" s="31" t="inlineStr">
+        <is>
+          <t>Hikvision</t>
+        </is>
+      </c>
+      <c r="D28" s="31" t="inlineStr">
+        <is>
+          <t>⚠️ No Recording Found</t>
+        </is>
+      </c>
+      <c r="E28" s="32" t="inlineStr">
+        <is>
+          <t>NVR reachable, no footage at this time</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="33" t="n">
+        <v>26</v>
+      </c>
+      <c r="B29" s="34" t="inlineStr">
+        <is>
+          <t>sgi-daanmogot</t>
+        </is>
+      </c>
+      <c r="C29" s="34" t="inlineStr">
+        <is>
+          <t>Hikvision</t>
+        </is>
+      </c>
+      <c r="D29" s="34" t="inlineStr">
+        <is>
+          <t>⚠️ No Recording Found</t>
+        </is>
+      </c>
+      <c r="E29" s="35" t="inlineStr">
+        <is>
+          <t>NVR reachable, no footage at this time</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="30" t="n">
+        <v>27</v>
+      </c>
+      <c r="B30" s="31" t="inlineStr">
+        <is>
+          <t>sig-bekasi-cibitung</t>
+        </is>
+      </c>
+      <c r="C30" s="31" t="inlineStr">
+        <is>
+          <t>Hikvision</t>
+        </is>
+      </c>
+      <c r="D30" s="31" t="inlineStr">
+        <is>
+          <t>⚠️ No Recording Found</t>
+        </is>
+      </c>
+      <c r="E30" s="32" t="inlineStr">
+        <is>
+          <t>NVR reachable, no footage at this time</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="33" t="n">
+        <v>28</v>
+      </c>
+      <c r="B31" s="34" t="inlineStr">
+        <is>
+          <t>head-office-jakarta</t>
+        </is>
+      </c>
+      <c r="C31" s="34" t="inlineStr">
+        <is>
+          <t>ACTi SNVR</t>
+        </is>
+      </c>
+      <c r="D31" s="34" t="inlineStr">
+        <is>
+          <t>⚠️ No Recording Found</t>
+        </is>
+      </c>
+      <c r="E31" s="35" t="inlineStr">
+        <is>
+          <t>ACTi search API works, no footage returned</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="30" t="n">
+        <v>29</v>
+      </c>
+      <c r="B32" s="31" t="inlineStr">
+        <is>
+          <t>sandana-adi-prakarsa</t>
+        </is>
+      </c>
+      <c r="C32" s="31" t="inlineStr">
+        <is>
+          <t>ACTi SNVR</t>
+        </is>
+      </c>
+      <c r="D32" s="31" t="inlineStr">
+        <is>
+          <t>⚠️ No Recording Found</t>
+        </is>
+      </c>
+      <c r="E32" s="32" t="inlineStr">
+        <is>
+          <t>ACTi search API works, no footage returned</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="33" t="n">
+        <v>30</v>
+      </c>
+      <c r="B33" s="34" t="inlineStr">
+        <is>
+          <t>sandana-baswara-gas</t>
+        </is>
+      </c>
+      <c r="C33" s="34" t="inlineStr">
+        <is>
+          <t>ACTi SNVR</t>
+        </is>
+      </c>
+      <c r="D33" s="34" t="inlineStr">
+        <is>
+          <t>⚠️ No Recording Found</t>
+        </is>
+      </c>
+      <c r="E33" s="35" t="inlineStr">
+        <is>
+          <t>ACTi search API works, no footage returned</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="30" t="n">
+        <v>31</v>
+      </c>
+      <c r="B34" s="31" t="inlineStr">
+        <is>
+          <t>sgi-batakan</t>
+        </is>
+      </c>
+      <c r="C34" s="31" t="inlineStr">
+        <is>
+          <t>ACTi SNVR</t>
+        </is>
+      </c>
+      <c r="D34" s="31" t="inlineStr">
+        <is>
+          <t>⚠️ No Recording Found</t>
+        </is>
+      </c>
+      <c r="E34" s="32" t="inlineStr">
+        <is>
+          <t>ACTi search API works, no footage returned</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="33" t="n">
+        <v>32</v>
+      </c>
+      <c r="B35" s="34" t="inlineStr">
+        <is>
+          <t>sgi-boyolali</t>
+        </is>
+      </c>
+      <c r="C35" s="34" t="inlineStr">
+        <is>
+          <t>ACTi SNVR</t>
+        </is>
+      </c>
+      <c r="D35" s="34" t="inlineStr">
+        <is>
+          <t>⚠️ No Recording Found</t>
+        </is>
+      </c>
+      <c r="E35" s="35" t="inlineStr">
+        <is>
+          <t>ACTi search API works, no footage returned</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="30" t="n">
+        <v>33</v>
+      </c>
+      <c r="B36" s="31" t="inlineStr">
+        <is>
+          <t>sgi-duri</t>
+        </is>
+      </c>
+      <c r="C36" s="31" t="inlineStr">
+        <is>
+          <t>ACTi SNVR</t>
+        </is>
+      </c>
+      <c r="D36" s="31" t="inlineStr">
+        <is>
+          <t>⚠️ No Recording Found</t>
+        </is>
+      </c>
+      <c r="E36" s="32" t="inlineStr">
+        <is>
+          <t>ACTi search API works, no footage returned</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="33" t="n">
+        <v>34</v>
+      </c>
+      <c r="B37" s="34" t="inlineStr">
+        <is>
+          <t>sgi-jambi</t>
+        </is>
+      </c>
+      <c r="C37" s="34" t="inlineStr">
+        <is>
+          <t>ACTi SNVR</t>
+        </is>
+      </c>
+      <c r="D37" s="34" t="inlineStr">
+        <is>
+          <t>⚠️ No Recording Found</t>
+        </is>
+      </c>
+      <c r="E37" s="35" t="inlineStr">
+        <is>
+          <t>ACTi search API works, no footage returned</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="30" t="n">
+        <v>35</v>
+      </c>
+      <c r="B38" s="31" t="inlineStr">
+        <is>
+          <t>sgi-klaten</t>
+        </is>
+      </c>
+      <c r="C38" s="31" t="inlineStr">
+        <is>
+          <t>ACTi SNVR</t>
+        </is>
+      </c>
+      <c r="D38" s="31" t="inlineStr">
+        <is>
+          <t>⚠️ No Recording Found</t>
+        </is>
+      </c>
+      <c r="E38" s="32" t="inlineStr">
+        <is>
+          <t>ACTi search API works, no footage returned</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="33" t="n">
+        <v>36</v>
+      </c>
+      <c r="B39" s="34" t="inlineStr">
+        <is>
+          <t>sgi-kudus</t>
+        </is>
+      </c>
+      <c r="C39" s="34" t="inlineStr">
+        <is>
+          <t>ACTi SNVR</t>
+        </is>
+      </c>
+      <c r="D39" s="34" t="inlineStr">
+        <is>
+          <t>⚠️ No Recording Found</t>
+        </is>
+      </c>
+      <c r="E39" s="35" t="inlineStr">
+        <is>
+          <t>ACTi search API works, no footage returned</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="30" t="n">
+        <v>37</v>
+      </c>
+      <c r="B40" s="31" t="inlineStr">
+        <is>
+          <t>sgi-kutai</t>
+        </is>
+      </c>
+      <c r="C40" s="31" t="inlineStr">
+        <is>
+          <t>ACTi SNVR</t>
+        </is>
+      </c>
+      <c r="D40" s="31" t="inlineStr">
+        <is>
+          <t>⚠️ No Recording Found</t>
+        </is>
+      </c>
+      <c r="E40" s="32" t="inlineStr">
+        <is>
+          <t>ACTi search API works, no footage returned</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="33" t="n">
+        <v>38</v>
+      </c>
+      <c r="B41" s="34" t="inlineStr">
+        <is>
+          <t>sgi-madiun</t>
+        </is>
+      </c>
+      <c r="C41" s="34" t="inlineStr">
+        <is>
+          <t>ACTi SNVR</t>
+        </is>
+      </c>
+      <c r="D41" s="34" t="inlineStr">
+        <is>
+          <t>⚠️ No Recording Found</t>
+        </is>
+      </c>
+      <c r="E41" s="35" t="inlineStr">
+        <is>
+          <t>ACTi search API works, no footage returned</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="30" t="n">
+        <v>39</v>
+      </c>
+      <c r="B42" s="31" t="inlineStr">
+        <is>
+          <t>sgi-magelang</t>
+        </is>
+      </c>
+      <c r="C42" s="31" t="inlineStr">
+        <is>
+          <t>ACTi SNVR</t>
+        </is>
+      </c>
+      <c r="D42" s="31" t="inlineStr">
+        <is>
+          <t>⚠️ No Recording Found</t>
+        </is>
+      </c>
+      <c r="E42" s="32" t="inlineStr">
+        <is>
+          <t>ACTi search API works, no footage returned</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="33" t="n">
+        <v>40</v>
+      </c>
+      <c r="B43" s="34" t="inlineStr">
+        <is>
+          <t>sgi-malang</t>
+        </is>
+      </c>
+      <c r="C43" s="34" t="inlineStr">
+        <is>
+          <t>ACTi SNVR</t>
+        </is>
+      </c>
+      <c r="D43" s="34" t="inlineStr">
+        <is>
+          <t>⚠️ No Recording Found</t>
+        </is>
+      </c>
+      <c r="E43" s="35" t="inlineStr">
+        <is>
+          <t>ACTi search API works, no footage returned</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="30" t="n">
+        <v>41</v>
+      </c>
+      <c r="B44" s="31" t="inlineStr">
+        <is>
+          <t>sgi-pier</t>
+        </is>
+      </c>
+      <c r="C44" s="31" t="inlineStr">
+        <is>
+          <t>ACTi SNVR</t>
+        </is>
+      </c>
+      <c r="D44" s="31" t="inlineStr">
+        <is>
+          <t>⚠️ No Recording Found</t>
+        </is>
+      </c>
+      <c r="E44" s="32" t="inlineStr">
+        <is>
+          <t>ACTi search API works, no footage returned</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="33" t="n">
+        <v>42</v>
+      </c>
+      <c r="B45" s="34" t="inlineStr">
+        <is>
+          <t>sgi-sibolga</t>
+        </is>
+      </c>
+      <c r="C45" s="34" t="inlineStr">
+        <is>
+          <t>ACTi SNVR</t>
+        </is>
+      </c>
+      <c r="D45" s="34" t="inlineStr">
+        <is>
+          <t>⚠️ No Recording Found</t>
+        </is>
+      </c>
+      <c r="E45" s="35" t="inlineStr">
+        <is>
+          <t>ACTi search API works, no footage returned</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="30" t="n">
+        <v>43</v>
+      </c>
+      <c r="B46" s="31" t="inlineStr">
+        <is>
+          <t>sgi-tuban</t>
+        </is>
+      </c>
+      <c r="C46" s="31" t="inlineStr">
+        <is>
+          <t>ACTi SNVR</t>
+        </is>
+      </c>
+      <c r="D46" s="31" t="inlineStr">
+        <is>
+          <t>⚠️ No Recording Found</t>
+        </is>
+      </c>
+      <c r="E46" s="32" t="inlineStr">
+        <is>
+          <t>ACTi search API works, no footage returned</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="33" t="n">
+        <v>44</v>
+      </c>
+      <c r="B47" s="34" t="inlineStr">
+        <is>
+          <t>sig-bandung</t>
+        </is>
+      </c>
+      <c r="C47" s="34" t="inlineStr">
+        <is>
+          <t>ACTi SNVR</t>
+        </is>
+      </c>
+      <c r="D47" s="34" t="inlineStr">
+        <is>
+          <t>⚠️ No Recording Found</t>
+        </is>
+      </c>
+      <c r="E47" s="35" t="inlineStr">
+        <is>
+          <t>ACTi search API works, no footage returned</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="30" t="n">
+        <v>45</v>
+      </c>
+      <c r="B48" s="31" t="inlineStr">
+        <is>
+          <t>sig-gorontalo</t>
+        </is>
+      </c>
+      <c r="C48" s="31" t="inlineStr">
+        <is>
+          <t>ACTi SNVR</t>
+        </is>
+      </c>
+      <c r="D48" s="31" t="inlineStr">
+        <is>
+          <t>⚠️ No Recording Found</t>
+        </is>
+      </c>
+      <c r="E48" s="32" t="inlineStr">
+        <is>
+          <t>ACTi search API works, no footage returned</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="33" t="n">
+        <v>46</v>
+      </c>
+      <c r="B49" s="34" t="inlineStr">
+        <is>
+          <t>sig-manado</t>
+        </is>
+      </c>
+      <c r="C49" s="34" t="inlineStr">
+        <is>
+          <t>ACTi SNVR</t>
+        </is>
+      </c>
+      <c r="D49" s="34" t="inlineStr">
+        <is>
+          <t>⚠️ No Recording Found</t>
+        </is>
+      </c>
+      <c r="E49" s="35" t="inlineStr">
+        <is>
+          <t>ACTi search API works, no footage returned</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="30" t="n">
+        <v>47</v>
+      </c>
+      <c r="B50" s="31" t="inlineStr">
+        <is>
+          <t>sig-pekanbaru</t>
+        </is>
+      </c>
+      <c r="C50" s="31" t="inlineStr">
+        <is>
+          <t>ACTi SNVR</t>
+        </is>
+      </c>
+      <c r="D50" s="31" t="inlineStr">
+        <is>
+          <t>⚠️ No Recording Found</t>
+        </is>
+      </c>
+      <c r="E50" s="32" t="inlineStr">
+        <is>
+          <t>ACTi search API works, no footage returned</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="33" t="n">
+        <v>48</v>
+      </c>
+      <c r="B51" s="34" t="inlineStr">
+        <is>
+          <t>sig-rungkut-sier</t>
+        </is>
+      </c>
+      <c r="C51" s="34" t="inlineStr">
+        <is>
+          <t>ACTi SNVR</t>
+        </is>
+      </c>
+      <c r="D51" s="34" t="inlineStr">
+        <is>
+          <t>⚠️ No Recording Found</t>
+        </is>
+      </c>
+      <c r="E51" s="35" t="inlineStr">
+        <is>
+          <t>ACTi search API works, no footage returned</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="30" t="n">
+        <v>49</v>
+      </c>
+      <c r="B52" s="31" t="inlineStr">
+        <is>
+          <t>sig-siantar</t>
+        </is>
+      </c>
+      <c r="C52" s="31" t="inlineStr">
+        <is>
+          <t>ACTi SNVR</t>
+        </is>
+      </c>
+      <c r="D52" s="31" t="inlineStr">
+        <is>
+          <t>⚠️ No Recording Found</t>
+        </is>
+      </c>
+      <c r="E52" s="32" t="inlineStr">
+        <is>
+          <t>ACTi search API works, no footage returned</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="33" t="n">
+        <v>50</v>
+      </c>
+      <c r="B53" s="34" t="inlineStr">
+        <is>
+          <t>sig-ternate</t>
+        </is>
+      </c>
+      <c r="C53" s="34" t="inlineStr">
+        <is>
+          <t>ACTi SNVR</t>
+        </is>
+      </c>
+      <c r="D53" s="34" t="inlineStr">
+        <is>
+          <t>⚠️ No Recording Found</t>
+        </is>
+      </c>
+      <c r="E53" s="35" t="inlineStr">
+        <is>
+          <t>ACTi search API works, no footage returned</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="36" t="n">
+        <v>51</v>
+      </c>
+      <c r="B54" s="37" t="inlineStr">
+        <is>
+          <t>ame-gudang-krian</t>
+        </is>
+      </c>
+      <c r="C54" s="37" t="inlineStr">
+        <is>
+          <t>Uniview</t>
+        </is>
+      </c>
+      <c r="D54" s="37" t="inlineStr">
+        <is>
+          <t>❌ API Not Supported</t>
+        </is>
+      </c>
+      <c r="E54" s="38" t="inlineStr">
+        <is>
+          <t>Missing /ISAPI/ContentMgmt/search — needs Uniview playback impl</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="39" t="n">
+        <v>52</v>
+      </c>
+      <c r="B55" s="40" t="inlineStr">
+        <is>
+          <t>sgi-bangka</t>
+        </is>
+      </c>
+      <c r="C55" s="40" t="inlineStr">
+        <is>
+          <t>Uniview</t>
+        </is>
+      </c>
+      <c r="D55" s="40" t="inlineStr">
+        <is>
+          <t>❌ API Not Supported</t>
+        </is>
+      </c>
+      <c r="E55" s="41" t="inlineStr">
+        <is>
+          <t>Missing /ISAPI/ContentMgmt/search — needs Uniview playback impl</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="A1:E1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>